<commit_message>
feat: updated Excel parsing to handle new layout with leading empty row
</commit_message>
<xml_diff>
--- a/public/SafirMed.xlsx
+++ b/public/SafirMed.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="200" uniqueCount="113">
   <si>
     <t>Spécialité</t>
   </si>
@@ -77,7 +77,7 @@
     <t>05 23 35 38 50</t>
   </si>
   <si>
-    <t>Ophtalmo</t>
+    <t>Ophtalmologie</t>
   </si>
   <si>
     <t>Dr. Amri Amine Jade</t>
@@ -143,7 +143,7 @@
     <t>06 20 46 36 62</t>
   </si>
   <si>
-    <t>Cardio</t>
+    <t>Cardiologie</t>
   </si>
   <si>
     <t>Dr. Abdelilah Bentalha</t>
@@ -207,6 +207,165 @@
   </si>
   <si>
     <t>05 23 35 35 22</t>
+  </si>
+  <si>
+    <t>Pédiatrie</t>
+  </si>
+  <si>
+    <t>Dr. Ghema Karima</t>
+  </si>
+  <si>
+    <t>05 23 35 01 00</t>
+  </si>
+  <si>
+    <t>Dr. Hasnaa Almiaadi</t>
+  </si>
+  <si>
+    <t>07 73 14 18 24</t>
+  </si>
+  <si>
+    <t>Dr. Ilham Bentalha</t>
+  </si>
+  <si>
+    <t>05 23 39 54 16</t>
+  </si>
+  <si>
+    <t>Dr. Benatiya Andaloussi Wiame</t>
+  </si>
+  <si>
+    <t>05 23 35 47 81</t>
+  </si>
+  <si>
+    <t>Dr. Fouad Nadia</t>
+  </si>
+  <si>
+    <t>06 62 25 62 30</t>
+  </si>
+  <si>
+    <t>Gastro-entérologie</t>
+  </si>
+  <si>
+    <t>Dr. Chaouch Safaa</t>
+  </si>
+  <si>
+    <t>05 23 39 04 99</t>
+  </si>
+  <si>
+    <t>Dr. Imane Korch</t>
+  </si>
+  <si>
+    <t>05 23 37 12 71</t>
+  </si>
+  <si>
+    <t>Dr. Lahlou Houda</t>
+  </si>
+  <si>
+    <t>05 23 38 78 92</t>
+  </si>
+  <si>
+    <t>Dr. Amina Bahbouhi</t>
+  </si>
+  <si>
+    <t>05 23 36 18 29</t>
+  </si>
+  <si>
+    <t>Dr. Toumi Najoua</t>
+  </si>
+  <si>
+    <t>07 04 83 29 97</t>
+  </si>
+  <si>
+    <t>Gynécologie</t>
+  </si>
+  <si>
+    <t>Dr. Hanane Laghmari</t>
+  </si>
+  <si>
+    <t>05 23 34 37 72</t>
+  </si>
+  <si>
+    <t>Dr. Sadi Marouane</t>
+  </si>
+  <si>
+    <t>05 23 33 62 88</t>
+  </si>
+  <si>
+    <t>Dr. Nabhani Mouna</t>
+  </si>
+  <si>
+    <t>05 23 33 68 68</t>
+  </si>
+  <si>
+    <t>Dr. Dounia Britel</t>
+  </si>
+  <si>
+    <t>05 23 34 47 98</t>
+  </si>
+  <si>
+    <t>Dr. Mohamed Said Abou Elfattah</t>
+  </si>
+  <si>
+    <t>05 23 37 30 31</t>
+  </si>
+  <si>
+    <t>Neurologie</t>
+  </si>
+  <si>
+    <t>Dr. Adil Aqqad</t>
+  </si>
+  <si>
+    <t>06 63 87 56 00</t>
+  </si>
+  <si>
+    <t>Dr. Kaddour Marfoq</t>
+  </si>
+  <si>
+    <t>05 23 39 19 99</t>
+  </si>
+  <si>
+    <t>Dr. Mohamed Jafoui</t>
+  </si>
+  <si>
+    <t>05 23 37 30 00</t>
+  </si>
+  <si>
+    <t>Dr. Abdelhaq Zaïm</t>
+  </si>
+  <si>
+    <t>05 23 39 31 55</t>
+  </si>
+  <si>
+    <t>Orthopédie</t>
+  </si>
+  <si>
+    <t>Dr. Guermal Abdelaziz</t>
+  </si>
+  <si>
+    <t>05 23 34 35 33</t>
+  </si>
+  <si>
+    <t>Dr. Mourad Zahiri</t>
+  </si>
+  <si>
+    <t>05 23 39 46 97</t>
+  </si>
+  <si>
+    <t>Dr. Amine Sdoudi</t>
+  </si>
+  <si>
+    <t>07 01 11 02 59</t>
+  </si>
+  <si>
+    <t>Dr. Mohamed Bayad</t>
+  </si>
+  <si>
+    <t>06 61 31 65 64</t>
+  </si>
+  <si>
+    <t>Dr. Mostafa El Bestani</t>
+  </si>
+  <si>
+    <t>06 62 11 43 83</t>
   </si>
 </sst>
 </file>
@@ -228,15 +387,15 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
+      <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
+      <b/>
+      <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
@@ -387,7 +546,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="33">
+  <fills count="43">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -396,6 +555,66 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFFF17DC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF67C551"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF61E1E9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDC7AFC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFACACAC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF6FF61"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF39F44F"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF73D3FF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFECA6F4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF3535FF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFFFFFCC"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -581,7 +800,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="22">
     <border>
       <left/>
       <right/>
@@ -590,16 +809,196 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
         <color auto="1"/>
       </left>
       <right style="thin">
         <color auto="1"/>
       </right>
-      <top style="thin">
+      <top style="medium">
         <color auto="1"/>
       </top>
       <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
         <color auto="1"/>
       </bottom>
       <diagonal/>
@@ -705,19 +1104,19 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -726,7 +1125,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="14" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -738,127 +1137,246 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="15" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="16" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="13" borderId="17" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="14" borderId="18" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="14" borderId="17" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="15" borderId="19" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="20" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="21" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="40" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="41" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="42" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="11" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="11" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -912,6 +1430,20 @@
     <cellStyle name="60 % - Accent6" xfId="48" builtinId="52"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="0061E1E9"/>
+      <color rgb="00DC7AFC"/>
+      <color rgb="00ACACAC"/>
+      <color rgb="00F6FF61"/>
+      <color rgb="0039F44F"/>
+      <color rgb="00C3FF31"/>
+      <color rgb="0073D3FF"/>
+      <color rgb="00ECA6F4"/>
+      <color rgb="000000E2"/>
+      <color rgb="003535FF"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -1178,383 +1710,716 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:D27"/>
+  <dimension ref="A1:D51"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelCol="3"/>
   <cols>
-    <col min="1" max="1" width="17.7777777777778" customWidth="1"/>
-    <col min="2" max="2" width="27.1111111111111" customWidth="1"/>
-    <col min="3" max="3" width="15" customWidth="1"/>
+    <col min="1" max="1" width="18.7777777777778" style="2" customWidth="1"/>
+    <col min="2" max="2" width="31.7777777777778" style="2" customWidth="1"/>
+    <col min="3" max="3" width="16.7777777777778" style="2" customWidth="1"/>
+    <col min="4" max="4" width="12.3333333333333" style="2" customWidth="1"/>
+    <col min="5" max="16384" width="9" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28.8" spans="1:4">
-      <c r="A1" s="1" t="s">
+    <row r="1" ht="15.15"/>
+    <row r="2" ht="28" customHeight="1" spans="1:4">
+      <c r="A2" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C2" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D2" s="3" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" ht="28.8" spans="1:4">
-      <c r="A2" s="2" t="s">
+    <row r="3" ht="15.6" spans="1:4">
+      <c r="A3" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B3" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C3" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="3" ht="43.2" spans="1:4">
-      <c r="A3" s="2" t="s">
+      <c r="D3" s="7" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" ht="15.6" spans="1:4">
+      <c r="A4" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B4" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C4" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="D3" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="4" ht="43.2" spans="1:4">
-      <c r="A4" s="2" t="s">
+      <c r="D4" s="11" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" ht="15.6" spans="1:4">
+      <c r="A5" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B5" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C5" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="D4" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="5" ht="43.2" spans="1:4">
-      <c r="A5" s="2" t="s">
+      <c r="D5" s="11" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" ht="15.6" spans="1:4">
+      <c r="A6" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B6" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C6" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="D5" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="6" ht="43.2" spans="1:4">
-      <c r="A6" s="2" t="s">
+      <c r="D6" s="11" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="7" ht="16.35" spans="1:4">
+      <c r="A7" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B7" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="C7" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="D6" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="7" ht="43.2" spans="1:4">
-      <c r="A7" s="2" t="s">
+      <c r="D7" s="15" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8" ht="15.6" spans="1:4">
+      <c r="A8" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B8" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="C8" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="D7" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="8" ht="28.8" spans="1:4">
-      <c r="A8" s="2" t="s">
+      <c r="D8" s="7" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" ht="15.6" spans="1:4">
+      <c r="A9" s="17" t="s">
         <v>16</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B9" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="C9" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="D8" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="9" ht="43.2" spans="1:4">
-      <c r="A9" s="2" t="s">
+      <c r="D9" s="11" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="10" ht="15.6" spans="1:4">
+      <c r="A10" s="17" t="s">
         <v>16</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B10" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="C10" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="D9" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="10" ht="28.8" spans="1:4">
-      <c r="A10" s="2" t="s">
+      <c r="D10" s="11" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="11" ht="15.6" spans="1:4">
+      <c r="A11" s="17" t="s">
         <v>16</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B11" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="C11" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="D10" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="11" ht="28.8" spans="1:4">
-      <c r="A11" s="2" t="s">
+      <c r="D11" s="11" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="12" ht="16.35" spans="1:4">
+      <c r="A12" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B12" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="C12" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="D11" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="12" ht="43.2" spans="1:4">
-      <c r="A12" s="2" t="s">
+      <c r="D12" s="15" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="13" ht="15.6" spans="1:4">
+      <c r="A13" s="19" t="s">
         <v>27</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B13" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="C13" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="D12" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="13" ht="43.2" spans="1:4">
-      <c r="A13" s="2" t="s">
+      <c r="D13" s="7" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="14" ht="15.6" spans="1:4">
+      <c r="A14" s="20" t="s">
         <v>27</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="B14" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="C13" s="2" t="s">
+      <c r="C14" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="D13" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="14" ht="43.2" spans="1:4">
-      <c r="A14" s="2" t="s">
+      <c r="D14" s="11" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="15" ht="15.6" spans="1:4">
+      <c r="A15" s="20" t="s">
         <v>27</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="B15" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="C14" s="2" t="s">
+      <c r="C15" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="D14" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="15" ht="43.2" spans="1:4">
-      <c r="A15" s="2" t="s">
+      <c r="D15" s="11" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="16" ht="15.6" spans="1:4">
+      <c r="A16" s="20" t="s">
         <v>27</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="B16" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="C15" s="2" t="s">
+      <c r="C16" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="D15" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="16" ht="57.6" spans="1:4">
-      <c r="A16" s="2" t="s">
+      <c r="D16" s="11" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="17" ht="16.35" spans="1:4">
+      <c r="A17" s="21" t="s">
         <v>27</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="B17" s="13" t="s">
         <v>36</v>
       </c>
-      <c r="C16" s="2" t="s">
+      <c r="C17" s="14" t="s">
         <v>37</v>
       </c>
-      <c r="D16" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="17" ht="43.2" spans="1:4">
-      <c r="A17" s="2" t="s">
+      <c r="D17" s="15" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="18" ht="15.6" spans="1:4">
+      <c r="A18" s="22" t="s">
         <v>38</v>
       </c>
-      <c r="B17" s="2" t="s">
+      <c r="B18" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="C17" s="2" t="s">
+      <c r="C18" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="D17" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="18" ht="28.8" spans="1:4">
-      <c r="A18" s="2" t="s">
+      <c r="D18" s="7" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="19" ht="15.6" spans="1:4">
+      <c r="A19" s="23" t="s">
         <v>38</v>
       </c>
-      <c r="B18" s="2" t="s">
+      <c r="B19" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="C18" s="2" t="s">
+      <c r="C19" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="D18" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="19" ht="43.2" spans="1:4">
-      <c r="A19" s="2" t="s">
+      <c r="D19" s="11" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="20" ht="15.6" spans="1:4">
+      <c r="A20" s="23" t="s">
         <v>38</v>
       </c>
-      <c r="B19" s="2" t="s">
+      <c r="B20" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="C19" s="2" t="s">
+      <c r="C20" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="D19" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="20" ht="43.2" spans="1:4">
-      <c r="A20" s="2" t="s">
+      <c r="D20" s="11" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="21" ht="15.6" spans="1:4">
+      <c r="A21" s="23" t="s">
         <v>38</v>
       </c>
-      <c r="B20" s="2" t="s">
+      <c r="B21" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="C20" s="2" t="s">
+      <c r="C21" s="10" t="s">
         <v>46</v>
       </c>
-      <c r="D20" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="21" ht="28.8" spans="1:4">
-      <c r="A21" s="2" t="s">
+      <c r="D21" s="11" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="22" ht="16.35" spans="1:4">
+      <c r="A22" s="24" t="s">
         <v>38</v>
       </c>
-      <c r="B21" s="2" t="s">
+      <c r="B22" s="13" t="s">
         <v>47</v>
       </c>
-      <c r="C21" s="2" t="s">
+      <c r="C22" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="D21" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="22" ht="28.8" spans="1:4">
-      <c r="A22" s="2" t="s">
+      <c r="D22" s="15" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="23" ht="15.6" spans="1:4">
+      <c r="A23" s="25" t="s">
         <v>49</v>
       </c>
-      <c r="B22" s="2" t="s">
+      <c r="B23" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="C22" s="2" t="s">
+      <c r="C23" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="D22" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="23" ht="28.8" spans="1:4">
-      <c r="A23" s="2" t="s">
+      <c r="D23" s="7" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="24" ht="15.6" spans="1:4">
+      <c r="A24" s="26" t="s">
         <v>49</v>
       </c>
-      <c r="B23" s="2" t="s">
+      <c r="B24" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="C23" s="2" t="s">
+      <c r="C24" s="10" t="s">
         <v>53</v>
       </c>
-      <c r="D23" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="24" ht="43.2" spans="1:4">
-      <c r="A24" s="2" t="s">
+      <c r="D24" s="11" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="25" ht="15.6" spans="1:4">
+      <c r="A25" s="26" t="s">
         <v>49</v>
       </c>
-      <c r="B24" s="2" t="s">
+      <c r="B25" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="C24" s="2" t="s">
+      <c r="C25" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="D24" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="25" ht="57.6" spans="1:4">
-      <c r="A25" s="2" t="s">
+      <c r="D25" s="11" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="26" ht="15.6" spans="1:4">
+      <c r="A26" s="26" t="s">
         <v>49</v>
       </c>
-      <c r="B25" s="2" t="s">
+      <c r="B26" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="C25" s="2" t="s">
+      <c r="C26" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="D25" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="26" ht="28.8" spans="1:4">
-      <c r="A26" s="2" t="s">
+      <c r="D26" s="11" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="27" ht="16.35" spans="1:4">
+      <c r="A27" s="27" t="s">
         <v>49</v>
       </c>
-      <c r="B26" s="2" t="s">
+      <c r="B27" s="13" t="s">
         <v>58</v>
       </c>
-      <c r="C26" s="2" t="s">
+      <c r="C27" s="14" t="s">
         <v>59</v>
       </c>
-      <c r="D26" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4">
-      <c r="A27" s="3"/>
-      <c r="B27" s="3"/>
-      <c r="C27" s="3"/>
-      <c r="D27" s="3"/>
+      <c r="D27" s="15" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="28" ht="15.6" spans="1:4">
+      <c r="A28" s="28" t="s">
+        <v>60</v>
+      </c>
+      <c r="B28" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="C28" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="D28" s="7" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="29" ht="15.6" spans="1:4">
+      <c r="A29" s="29" t="s">
+        <v>60</v>
+      </c>
+      <c r="B29" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="C29" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="D29" s="11" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="30" ht="15.6" spans="1:4">
+      <c r="A30" s="29" t="s">
+        <v>60</v>
+      </c>
+      <c r="B30" s="9" t="s">
+        <v>65</v>
+      </c>
+      <c r="C30" s="10" t="s">
+        <v>66</v>
+      </c>
+      <c r="D30" s="11" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="31" s="1" customFormat="1" ht="15.6" spans="1:4">
+      <c r="A31" s="29" t="s">
+        <v>60</v>
+      </c>
+      <c r="B31" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="C31" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="D31" s="11" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="32" ht="16.35" spans="1:4">
+      <c r="A32" s="30" t="s">
+        <v>60</v>
+      </c>
+      <c r="B32" s="13" t="s">
+        <v>69</v>
+      </c>
+      <c r="C32" s="14" t="s">
+        <v>70</v>
+      </c>
+      <c r="D32" s="15" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="33" ht="15.6" spans="1:4">
+      <c r="A33" s="31" t="s">
+        <v>71</v>
+      </c>
+      <c r="B33" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="C33" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="D33" s="7" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="34" ht="15.6" spans="1:4">
+      <c r="A34" s="32" t="s">
+        <v>71</v>
+      </c>
+      <c r="B34" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="C34" s="10" t="s">
+        <v>75</v>
+      </c>
+      <c r="D34" s="11" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="35" ht="15.6" spans="1:4">
+      <c r="A35" s="32" t="s">
+        <v>71</v>
+      </c>
+      <c r="B35" s="9" t="s">
+        <v>76</v>
+      </c>
+      <c r="C35" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="D35" s="11" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="36" ht="15.6" spans="1:4">
+      <c r="A36" s="32" t="s">
+        <v>71</v>
+      </c>
+      <c r="B36" s="9" t="s">
+        <v>78</v>
+      </c>
+      <c r="C36" s="10" t="s">
+        <v>79</v>
+      </c>
+      <c r="D36" s="11" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="37" ht="16.35" spans="1:4">
+      <c r="A37" s="33" t="s">
+        <v>71</v>
+      </c>
+      <c r="B37" s="13" t="s">
+        <v>80</v>
+      </c>
+      <c r="C37" s="14" t="s">
+        <v>81</v>
+      </c>
+      <c r="D37" s="15" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="38" ht="15.6" spans="1:4">
+      <c r="A38" s="34" t="s">
+        <v>82</v>
+      </c>
+      <c r="B38" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="C38" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="D38" s="7" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="39" ht="15.6" spans="1:4">
+      <c r="A39" s="35" t="s">
+        <v>82</v>
+      </c>
+      <c r="B39" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="C39" s="10" t="s">
+        <v>86</v>
+      </c>
+      <c r="D39" s="11" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="40" ht="15.6" spans="1:4">
+      <c r="A40" s="35" t="s">
+        <v>82</v>
+      </c>
+      <c r="B40" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="C40" s="10" t="s">
+        <v>88</v>
+      </c>
+      <c r="D40" s="11" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="41" ht="15.6" spans="1:4">
+      <c r="A41" s="35" t="s">
+        <v>82</v>
+      </c>
+      <c r="B41" s="9" t="s">
+        <v>89</v>
+      </c>
+      <c r="C41" s="10" t="s">
+        <v>90</v>
+      </c>
+      <c r="D41" s="11" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="42" s="1" customFormat="1" ht="16.35" spans="1:4">
+      <c r="A42" s="36" t="s">
+        <v>82</v>
+      </c>
+      <c r="B42" s="13" t="s">
+        <v>91</v>
+      </c>
+      <c r="C42" s="14" t="s">
+        <v>92</v>
+      </c>
+      <c r="D42" s="15" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="43" ht="15.6" spans="1:4">
+      <c r="A43" s="37" t="s">
+        <v>93</v>
+      </c>
+      <c r="B43" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="C43" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="D43" s="7" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="44" ht="15.6" spans="1:4">
+      <c r="A44" s="38" t="s">
+        <v>93</v>
+      </c>
+      <c r="B44" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="C44" s="10" t="s">
+        <v>97</v>
+      </c>
+      <c r="D44" s="11" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="45" ht="15.6" spans="1:4">
+      <c r="A45" s="38" t="s">
+        <v>93</v>
+      </c>
+      <c r="B45" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="C45" s="10" t="s">
+        <v>99</v>
+      </c>
+      <c r="D45" s="11" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="46" ht="16.35" spans="1:4">
+      <c r="A46" s="39" t="s">
+        <v>93</v>
+      </c>
+      <c r="B46" s="13" t="s">
+        <v>100</v>
+      </c>
+      <c r="C46" s="14" t="s">
+        <v>101</v>
+      </c>
+      <c r="D46" s="15" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="47" ht="15.6" spans="1:4">
+      <c r="A47" s="40" t="s">
+        <v>102</v>
+      </c>
+      <c r="B47" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="C47" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="D47" s="7" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="48" ht="15.6" spans="1:4">
+      <c r="A48" s="41" t="s">
+        <v>102</v>
+      </c>
+      <c r="B48" s="9" t="s">
+        <v>105</v>
+      </c>
+      <c r="C48" s="10" t="s">
+        <v>106</v>
+      </c>
+      <c r="D48" s="11" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="49" ht="15.6" spans="1:4">
+      <c r="A49" s="41" t="s">
+        <v>102</v>
+      </c>
+      <c r="B49" s="9" t="s">
+        <v>107</v>
+      </c>
+      <c r="C49" s="10" t="s">
+        <v>108</v>
+      </c>
+      <c r="D49" s="11" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="50" ht="15.6" spans="1:4">
+      <c r="A50" s="41" t="s">
+        <v>102</v>
+      </c>
+      <c r="B50" s="9" t="s">
+        <v>109</v>
+      </c>
+      <c r="C50" s="10" t="s">
+        <v>110</v>
+      </c>
+      <c r="D50" s="11" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="51" ht="16.35" spans="1:4">
+      <c r="A51" s="42" t="s">
+        <v>102</v>
+      </c>
+      <c r="B51" s="13" t="s">
+        <v>111</v>
+      </c>
+      <c r="C51" s="14" t="s">
+        <v>112</v>
+      </c>
+      <c r="D51" s="15" t="s">
+        <v>7</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>